<commit_message>
Updated timeline bar chart
</commit_message>
<xml_diff>
--- a/data/Research Papers.xlsx
+++ b/data/Research Papers.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ljaljevi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74241B7C-A71A-4B60-B204-E806CCE1BCFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16B4DB7-6B2C-4892-87CC-AAB4602317AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{027DABDA-E301-6248-9EF5-B2B8807799A0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{027DABDA-E301-6248-9EF5-B2B8807799A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="268">
   <si>
     <t>Title</t>
   </si>
@@ -1333,9 +1333,6 @@
   </si>
   <si>
     <t>Tomer Bitan and Tal Kadosh and Erel Kaplan and Shira Meiri and Le Chen and Peter Morales and Niranjan Hasabnis and Gal Oren</t>
-  </si>
-  <si>
-    <t>2026</t>
   </si>
 </sst>
 </file>
@@ -1456,7 +1453,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1492,6 +1489,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1727,28 +1727,6 @@
             </c:extLst>
           </c:dPt>
           <c:dLbls>
-            <c:dLbl>
-              <c:idx val="3"/>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="0"/>
-                  <c:y val="6.685510405806129E-2"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:dLblPos val="outEnd"/>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000000-EA81-4FD4-8DBD-4FC885948BA9}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -1805,9 +1783,9 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Timeline Main Research'!$D$9:$D$13</c:f>
+              <c:f>'Timeline Main Research'!$D$9:$D$12</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>2023</c:v>
                 </c:pt>
@@ -1817,18 +1795,15 @@
                 <c:pt idx="2">
                   <c:v>2025</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>2026</c:v>
-                </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Timeline Main Research'!$E$9:$E$13</c:f>
+              <c:f>'Timeline Main Research'!$E$9:$E$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>3</c:v>
                 </c:pt>
@@ -1836,10 +1811,7 @@
                   <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2643,9 +2615,9 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Ljaljevic, Strahinja" refreshedDate="46141.403660532407" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="28" xr:uid="{7E58EB42-7530-3042-8255-3A940C0AEDDC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Ljaljevic, Strahinja" refreshedDate="46153.435911111112" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="32" xr:uid="{D2FCC20E-3010-47C7-980A-7F2517E1B2F8}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:G29" sheet="Raw Main Research"/>
+    <worksheetSource ref="A1:G33" sheet="Raw Main Research"/>
   </cacheSource>
   <cacheFields count="9">
     <cacheField name="Title" numFmtId="0">
@@ -2658,7 +2630,7 @@
       <sharedItems longText="1"/>
     </cacheField>
     <cacheField name="Year" numFmtId="164">
-      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2023-09-01T00:00:00" maxDate="2026-01-26T00:00:00" count="33">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2023-09-01T00:00:00" maxDate="2025-12-23T00:00:00" count="27">
         <d v="2024-02-01T00:00:00"/>
         <d v="2024-05-01T00:00:00"/>
         <d v="2023-10-01T00:00:00"/>
@@ -2677,21 +2649,15 @@
         <d v="2025-06-01T00:00:00"/>
         <d v="2024-12-27T00:00:00"/>
         <d v="2025-11-15T00:00:00"/>
-        <d v="2026-01-25T00:00:00"/>
+        <d v="2025-12-01T00:00:00"/>
         <d v="2025-11-09T00:00:00"/>
         <d v="2025-05-04T00:00:00"/>
         <d v="2025-12-18T00:00:00"/>
         <d v="2025-10-30T00:00:00"/>
         <d v="2025-12-22T00:00:00"/>
-        <d v="2023-11-01T00:00:00" u="1"/>
-        <d v="2023-12-01T00:00:00" u="1"/>
-        <d v="2024-01-01T00:00:00" u="1"/>
-        <d v="2024-03-01T00:00:00" u="1"/>
-        <d v="2024-04-01T00:00:00" u="1"/>
-        <d v="2024-06-01T00:00:00" u="1"/>
-        <d v="2024-07-01T00:00:00" u="1"/>
-        <d v="2024-09-01T00:00:00" u="1"/>
-        <d v="2024-10-01T00:00:00" u="1"/>
+        <d v="2025-09-29T00:00:00"/>
+        <d v="2025-07-23T00:00:00"/>
+        <d v="2025-09-15T00:00:00"/>
       </sharedItems>
       <fieldGroup par="8"/>
     </cacheField>
@@ -2706,7 +2672,7 @@
     </cacheField>
     <cacheField name="Months (Year)" numFmtId="0" databaseField="0">
       <fieldGroup base="3">
-        <rangePr groupBy="months" startDate="2023-09-01T00:00:00" endDate="2026-01-26T00:00:00"/>
+        <rangePr groupBy="months" startDate="2023-09-01T00:00:00" endDate="2025-12-23T00:00:00"/>
         <groupItems count="14">
           <s v="&lt;9/1/2023"/>
           <s v="Jan"/>
@@ -2721,20 +2687,19 @@
           <s v="Oct"/>
           <s v="Nov"/>
           <s v="Dec"/>
-          <s v="&gt;1/26/2026"/>
+          <s v="&gt;12/23/2025"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
     <cacheField name="Years (Year)" numFmtId="0" databaseField="0">
       <fieldGroup base="3">
-        <rangePr groupBy="years" startDate="2023-09-01T00:00:00" endDate="2026-01-26T00:00:00"/>
-        <groupItems count="6">
+        <rangePr groupBy="years" startDate="2023-09-01T00:00:00" endDate="2025-12-23T00:00:00"/>
+        <groupItems count="5">
           <s v="&lt;9/1/2023"/>
           <s v="2023"/>
           <s v="2024"/>
           <s v="2025"/>
-          <s v="2026"/>
-          <s v="&gt;1/26/2026"/>
+          <s v="&gt;12/23/2025"/>
         </groupItems>
       </fieldGroup>
     </cacheField>
@@ -2748,7 +2713,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="28">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="32">
   <r>
     <s v="The Landscape and Challenges of HPC Research and LLMs"/>
     <s v="chen_landscape_2024"/>
@@ -3001,32 +2966,59 @@
     <s v="Y"/>
     <s v="Parallelization &amp; Optimization, Frameworks &amp; Architectures"/>
   </r>
+  <r>
+    <s v="Chat{PORT}: Fine-Tuned {LLM} for Easy Code {PORT}ing"/>
+    <s v="Pophale2026ChatPORT"/>
+    <s v="Swaroop Pophale and Zheming Jin and Keita Teranishi"/>
+    <x v="24"/>
+    <s v="Main Research Paper"/>
+    <s v="Y"/>
+    <s v="Code Generation, Frameworks &amp; Architectures"/>
+  </r>
+  <r>
+    <s v="Enhancing Chat{PORT} with {CUDA}-to-{SYCL} Kernel Translation Capability"/>
+    <s v="Jin2025ChatPORTCudaSyCL"/>
+    <s v="Zheming Jin and Swaroop Pophale and Keita Teranishi"/>
+    <x v="17"/>
+    <s v="Main Research Paper"/>
+    <s v="Y"/>
+    <s v="Code Generation, Frameworks &amp; Architectures"/>
+  </r>
+  <r>
+    <s v="{PCEBench}: A Multi-Dimensional Benchmark for Evaluating Large Language Models in Parallel Code Generation"/>
+    <s v="Chen2025PCEBench"/>
+    <s v="L. Chen and N. Ahmed and M. Capot{\u{a}} and T. Willke and N. Hasabnis and A. Jannesari"/>
+    <x v="25"/>
+    <s v="Main Research Paper"/>
+    <s v="Y"/>
+    <s v="Evaluation &amp; Benchmarking"/>
+  </r>
+  <r>
+    <s v="{UniPar}: A Unified LLM-Based Framework for Parallel and Accelerated Code Translation in {HPC}"/>
+    <s v="Bitan2025UniPar"/>
+    <s v="Tomer Bitan and Tal Kadosh and Erel Kaplan and Shira Meiri and Le Chen and Peter Morales and Niranjan Hasabnis and Gal Oren"/>
+    <x v="26"/>
+    <s v="Main Research Paper"/>
+    <s v="Y"/>
+    <s v="Code Generation, Frameworks &amp; Architectures"/>
+  </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6AC5E488-DAC0-1B46-86E0-729BAED744A6}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="28">
-  <location ref="D8:E13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7DEE0883-C0F8-4128-94F6-E3020B8D5509}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34">
+  <location ref="D8:E12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField numFmtId="164" showAll="0">
-      <items count="34">
+      <items count="28">
         <item x="7"/>
         <item x="2"/>
-        <item m="1" x="24"/>
-        <item m="1" x="25"/>
-        <item m="1" x="26"/>
         <item x="0"/>
-        <item m="1" x="27"/>
-        <item m="1" x="28"/>
         <item x="1"/>
-        <item m="1" x="29"/>
-        <item m="1" x="30"/>
         <item x="6"/>
-        <item m="1" x="31"/>
-        <item m="1" x="32"/>
         <item x="5"/>
         <item x="4"/>
         <item x="10"/>
@@ -3040,12 +3032,15 @@
         <item x="15"/>
         <item x="16"/>
         <item x="17"/>
-        <item x="18"/>
         <item x="19"/>
         <item x="20"/>
         <item x="21"/>
         <item x="22"/>
         <item x="23"/>
+        <item x="18"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -3072,13 +3067,12 @@
       </items>
     </pivotField>
     <pivotField axis="axisRow" showAll="0">
-      <items count="7">
+      <items count="6">
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
         <item x="0"/>
         <item x="4"/>
-        <item x="5"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -3086,7 +3080,7 @@
   <rowFields count="1">
     <field x="8"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="4">
     <i>
       <x/>
     </i>
@@ -3095,9 +3089,6 @@
     </i>
     <i>
       <x v="2"/>
-    </i>
-    <i>
-      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -3109,7 +3100,7 @@
   <dataFields count="1">
     <dataField name="Count of Title" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="3">
+  <chartFormats count="2">
     <chartFormat chart="2" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -3124,18 +3115,6 @@
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="8" format="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="8" count="1" selected="0">
-            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
@@ -5296,7 +5275,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="15" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -5319,7 +5298,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B4" s="11" t="s">
@@ -5342,7 +5321,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="15" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="11" t="s">
@@ -5365,7 +5344,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="15" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="11" t="s">
@@ -5388,7 +5367,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="15" t="s">
         <v>45</v>
       </c>
       <c r="B7" s="11" t="s">
@@ -5411,7 +5390,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="15" t="s">
         <v>76</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -5434,7 +5413,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="15" t="s">
         <v>98</v>
       </c>
       <c r="B9" s="11" t="s">
@@ -5457,7 +5436,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="15" t="s">
         <v>100</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -5480,7 +5459,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="15" t="s">
         <v>102</v>
       </c>
       <c r="B11" s="11" t="s">
@@ -5503,7 +5482,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="15" t="s">
         <v>104</v>
       </c>
       <c r="B12" s="11" t="s">
@@ -5526,7 +5505,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="15" t="s">
         <v>107</v>
       </c>
       <c r="B13" s="11" t="s">
@@ -5549,7 +5528,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="15" t="s">
         <v>109</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -5572,7 +5551,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="15" t="s">
         <v>112</v>
       </c>
       <c r="B15" s="11" t="s">
@@ -5595,7 +5574,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="15" t="s">
         <v>150</v>
       </c>
       <c r="B16" s="11" t="s">
@@ -5618,7 +5597,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>202</v>
       </c>
       <c r="B17" s="11" t="s">
@@ -5641,7 +5620,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="15" t="s">
         <v>204</v>
       </c>
       <c r="B18" s="11" t="s">
@@ -5664,7 +5643,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="15" t="s">
         <v>207</v>
       </c>
       <c r="B19" s="11" t="s">
@@ -6028,7 +6007,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A4EE84F-C795-3E47-86D0-27A4DA3A3887}">
-  <dimension ref="D8:E13"/>
+  <dimension ref="D8:E12"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="12.75" bestFit="1" customWidth="1"/>
@@ -6083,23 +6062,15 @@
         <v>224</v>
       </c>
       <c r="E11">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D12" s="5" t="s">
-        <v>268</v>
+        <v>95</v>
       </c>
       <c r="E12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="4:5" x14ac:dyDescent="0.25">
-      <c r="D13" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="E13">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>